<commit_message>
docs: correct BT2 source attribution and strengthen validation plan
</commit_message>
<xml_diff>
--- a/tai-lieu/cd-phong/tuan-1/bt2-vong-tay-mau-co-san/BT2_CD_PHONG_Phu_luc_bang_chung.xlsx
+++ b/tai-lieu/cd-phong/tuan-1/bt2-vong-tay-mau-co-san/BT2_CD_PHONG_Phu_luc_bang_chung.xlsx
@@ -12,15 +12,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giá đối thủ theo nhóm" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Truy vết bằng chứng" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kế hoạch tuần 2" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phiếu tuần 2 CHƯA ĐIỀN" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Câu hỏi &amp; quyết định" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phiếu khách T2 CHƯA ĐIỀN" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đơn T2 CHƯA ĐIỀN" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm cần xác nhận" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Đọc trước'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Khảo sát trích nguồn'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Đọc trước'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Khảo sát trích nguồn'!$A$1:$F$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Giá đối thủ theo nhóm'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Truy vết bằng chứng'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Kế hoạch tuần 2'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Phiếu tuần 2 CHƯA ĐIỀN'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Câu hỏi &amp; quyết định'!$A$1:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Phiếu khách T2 CHƯA ĐIỀN'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Đơn T2 CHƯA ĐIỀN'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Điểm cần xác nhận'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -502,48 +508,60 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Bản tổng hợp 28 phản hồi ngày 18–19/10/2026 và các URL nhóm dẫn; chưa đối soát phản hồi gốc hoặc trang giá trực tuyến.</t>
+          <t>Các số được trích từ tệp nhóm cung cấp. Bản rà soát ngày 20/10 không phải lượt thu thêm dữ liệu: mốc khảo sát và ngày tra cứu giá vẫn giữ theo nguồn 18–19/10/2026. Chưa có đối soát phản hồi gốc hoặc kiểm tra lại trang giá trực tuyến.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="85" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Không có dữ liệu giả</t>
+          <t>Vướng mắc nguồn giá</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tab Phiếu tuần 2 chỉ có tiêu đề, chưa có dòng trả lời. Không thêm số đơn, doanh số, lợi nhuận, chỉ tiêu hoặc thời điểm chưa được chốt.</t>
+          <t>Tên Pinky gắn với hai domain trong bản nhóm; chưa xác minh URL/cấu hình tương ứng mức 30.000/50.000đ. Ba mẫu Imoon là một shop, không phải ba đối thủ độc lập.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="85" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Đếm mô tả</t>
+          <t>Biểu mẫu chưa có dữ liệu</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>269 từ theo khoảng trắng; đủ 200–300 từ.</t>
+          <t>Phiếu khách và bảng đơn tuần 2 chỉ có tiêu đề. Không thêm số thực; số người, số đơn và số chiếc được tách riêng.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="85" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Đếm mô tả</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>270 từ theo khoảng trắng; đủ 200–300 từ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>Bản gốc</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>De_xuat_va_danh_gia_hai_y_tuong_kinh_doanh.docx; SHA256: cda814302b50241543bf5dfcf63e5c608c0db47abc820c61412dd6ade8293065</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -554,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -933,8 +951,208 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="85" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Trong nhóm mua quà: thích kiểu đơn giản</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>64,3%</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Sở thích – cột A</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ thuộc nhóm mua quà; không dùng mẫu số 28 cho tỷ lệ 64,3%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="85" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Trong nhóm đeo hằng ngày: thích kiểu đơn giản</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>66,7%</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Sở thích – cột B</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Không suy ra mọi người mua để đeo đều thích mẫu của nhóm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="85" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm mua quà: ưu tiên Shopee</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Kênh mua ưu tiên – cột A</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Kênh ưu tiên, không phải lịch sử giao dịch. Nguồn không nêu tỷ lệ riêng ở dòng này.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="85" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Nhóm mua quà: ưu tiên cửa hàng/gian hàng trực tiếp</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Kênh mua ưu tiên – cột A</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Không suy rộng thành thị phần; các kênh được trích chưa bao quát mọi phản hồi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="85" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm mua quà: ưu tiên TikTok Shop</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Kênh mua ưu tiên – cột A</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Không mặc định nhóm đã mở hoặc có thể bán trên TikTok Shop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="85" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Nhóm đeo hằng ngày: ưu tiên cửa hàng/gian hàng trực tiếp</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Kênh mua ưu tiên – cột B</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Kênh ưu tiên, chưa phải nơi từng mua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="85" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm đeo hằng ngày: ưu tiên Shopee</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Kênh mua ưu tiên – cột B</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Không suy ra mức phí sàn hoặc quyết định mở shop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="85" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Nhóm đeo hằng ngày: ưu tiên Facebook/Instagram</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Mục 2.1, bảng chân dung, dòng Kênh mua ưu tiên – cột B</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Phân biệt kênh tiếp cận/tư vấn với kênh khách muốn giao dịch.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F13"/>
+  <autoFilter ref="A1:F21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -979,22 +1197,22 @@
     <row r="2" ht="85" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pinky Shop – vòng tay handmade</t>
+          <t>Giá được tài liệu ghi dưới tên “Pinky Shop” – cần xác minh tên/URL</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>30.000đ/chiếc; 50.000đ/bộ 2 theo mô tả; ô giá 50.000đ cần làm rõ</t>
+          <t>30.000đ/chiếc; 50.000đ/bộ 2 là số trong báo cáo, chưa gắn chắc với trang/mẫu</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Website người bán, theo ghi nhận của nhóm ngày 19/10/2026 [MC-02]</t>
+          <t>MC-00: bảng website đầu tài liệu dẫn quatanglambangtay.com; bảng đối thủ sau đó dẫn pinky.vn [MC-02]</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Có thể tham khảo mức giá, cách trình bày và dịch vụ. Không mặc định giá/cấu hình còn hiệu lực.</t>
+          <t>Hai tên miền khác nhau, chưa biết cùng đơn vị hay giá ứng với URL nào. Ô giá 50.000đ và giá mô tả cũng cần đối chiếu. Không dùng để chốt giá bán của nhóm.</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1393,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Giá đối thủ Pinky Shop</t>
+          <t>Giá tham khảo gắn tên Pinky – chưa xác định URL tương ứng</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bảng đối thủ trong MC-00 ghi kiểm tra ngày 19/10/2026</t>
+          <t>MC-00: bảng website ở phần 1.1 và bảng “Phương án 2: Vòng tay mẫu có sẵn”; thời điểm nhóm ghi là 19/10/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1190,7 +1408,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Trích theo nhóm; chưa kiểm lại trang trực tuyến. Giá mô tả và ô giá chưa thống nhất, cần xác nhận cấu hình.</t>
+          <t>Bảng đầu dẫn quatanglambangtay.com; bảng sau dẫn https://www.pinky.vn/products/vong-tay-vong-tay-nam-vong-tay-doi-ca-tinh-cuc-dep-ma-vdtcnn1. Chưa xác minh cùng đơn vị hoặc giá thuộc trang nào. Giữ 30.000/50.000đ như số được báo cáo, chưa coi là giá đã kiểm tra.</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1518,7 @@
     <row r="2" ht="85" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận nguồn hàng trước test</t>
+          <t>Xác nhận nguồn hàng trước thử bán</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1310,24 +1528,24 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Chốt thông tin mẫu có thể mua, chất liệu, cỡ, giá ở lượng mua thực, tồn hàng và phí giao. Nếu dùng ảnh shop phải ghi rõ nguồn, chưa gọi là ảnh mẫu của nhóm.</t>
+          <t>Chốt mẫu, thông tin chất liệu/cỡ có căn cứ, giá đơn nhỏ, tồn hàng, vận chuyển và điều kiện lỗi/đổi. Kiểm tra điều kiện sỉ thay vì coi giá tham khảo là báo giá.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Báo giá/trao đổi có ngày; ảnh có nguồn; cấu hình và điều kiện mua được shop xác nhận.</t>
+          <t>Báo giá/trao đổi có ngày, mẫu và lượng mua; phân biệt ảnh shop với ảnh do nhóm chụp.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Chưa có báo giá đơn nhỏ hoặc mẫu cuối được xác nhận trong đầu vào.</t>
+          <t>Chưa được cung cấp báo giá đơn nhỏ hoặc mẫu cuối được xác nhận.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="85" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Cho khách xem mẫu và hỏi nhu cầu</t>
+          <t>Hỏi trải nghiệm trước khi cho xem giá</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1337,24 +1555,24 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Tiếp cận 5–10 khách tiềm năng theo gợi ý của đề; hỏi mục đích, lựa chọn mẫu, cỡ/chất liệu quan tâm, mức giá chấp nhận và lý do từ chối. Ghi rõ người từng tham gia khảo sát cũ nếu khảo sát lại.</t>
+          <t>Đề xuất 5–10 khách theo gợi ý của đề. Hỏi lần mua vòng gần nhất, nơi mua, số tiền/đơn vị, mục đích, trở ngại và ngân sách trước khi đưa mẫu/giá để hạn chế dẫn dắt.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Phiếu theo mã người tham gia, thời điểm, mẫu/giá đã xem, câu trả lời; xin phép ghi nhận.</t>
+          <t>Mã người, ngày, cách tuyển, lần đầu/khảo sát lại, câu trả lời nguyên ý; cho phép chưa từng mua/không nhớ.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Cỡ mẫu này là kế hoạch kiểm chứng, không phải phản hồi đã thu.</t>
+          <t>Chưa có phản hồi tuần 2 được cung cấp; không điền thay khách.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="85" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra đề xuất giá trị</t>
+          <t>Cho xem cùng bộ thông tin và so sánh</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1364,17 +1582,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Cho khách xem ảnh/thông tin cụ thể và phương án tương tự; hỏi lý do chọn nhóm hoặc chọn nơi khác, không gợi ý câu trả lời.</t>
+          <t>Công bố đúng mẫu, nguồn ảnh, chất liệu/cỡ đã xác nhận, giá và phí nhận hàng. Hỏi chọn mẫu nào hoặc không chọn, vì sao, chọn nhóm hay nơi khác.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Ghi nguyên ý kiến về mẫu, chất liệu, giá, cách nhận; nguồn và giá đối thủ cùng thời điểm/cấu hình khi có.</t>
+          <t>Lưu phiên bản ảnh/mẫu, giá đã xem và lý do; nếu đổi mẫu/giá thì ghi riêng để tránh gộp kết quả khác điều kiện.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Không ghi nhóm vượt trội nếu chỉ là nhận xét nội bộ.</t>
+          <t>Có thể hỏi sở thích bằng ảnh shop ghi nguồn; chỉ nhận đơn khi có khả năng thực hiện.</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1609,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Chỉ công bố điều kiện có thể thực hiện; ghi riêng hỏi giá, quan tâm, xác nhận đặt, cọc, giao, hủy. Không thu cọc khi nhóm chưa thống nhất khả năng thực hiện và điều kiện giao dịch.</t>
+          <t>Ghi riêng quan tâm, xác nhận đặt, cọc, giao, hủy; gắn mã đơn và thời điểm. Không mặc định thu cọc hoặc đã mở shop sàn khi nhóm chưa thống nhất.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Mã đơn, mẫu/giá, thời điểm, trạng thái và chứng từ nếu phát sinh; ẩn thông tin riêng ở bản nộp.</t>
+          <t>Bảng đơn thật; số chiếc, giá, phí và chứng từ khi phát sinh; không đếm một khách hỏi nhiều lần thành nhiều khách.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Chưa có số đơn, tỷ lệ chuyển đổi hoặc doanh thu để báo cáo.</t>
+          <t>Phân biệt số người, số đơn và số chiếc; chưa có số thực để báo cáo.</t>
         </is>
       </c>
     </row>
@@ -1418,17 +1636,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Đối chiếu lựa chọn, lý do từ chối, mức giá, nguồn hàng và hành động mua. Giữ mẫu, sửa đề xuất hoặc thử tiếp dựa trên dữ liệu thu được.</t>
+          <t>Đối chiếu nhu cầu, mức giá, khả năng cung ứng và hành động thực. Phân loại giữ mẫu để thử tiếp, cần sửa hoặc chưa đủ căn cứ theo tiêu chí ở dưới.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Bảng kết quả thực; minh chứng nguồn; biên bản quyết định có người/ngày xác nhận.</t>
+          <t>Bảng kết quả có nguồn, phản hồi từ chối; quyết định ghi người/ngày và lý do.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Chưa tự đặt ngưỡng đạt, chỉ tiêu doanh số hoặc lịch ngày khi nhóm chưa chốt.</t>
+          <t>Các đầu mối/tiêu chí này là đề xuất, cần nhóm xác nhận trước triển khai.</t>
         </is>
       </c>
     </row>
@@ -1444,22 +1662,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="125" customWidth="1" min="2" max="2"/>
+    <col width="105" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Thời điểm / tình huống</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Câu hỏi / căn cứ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cách ghi nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="85" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Trước khi xem mẫu/giá</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Bạn đã từng mua vòng tay chưa? Lần gần nhất khi nào, ở đâu, trả bao nhiêu cho một chiếc/bộ?</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Cho phép chưa từng mua/không nhớ; ghi rõ đơn vị và giá tự khai, không bắt buộc chứng từ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="85" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Trước khi xem mẫu/giá</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Bạn mua để làm gì? Điều gì khiến bạn chọn hoặc bỏ mua? Ngân sách cho lần mua tới khoảng bao nhiêu?</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Ghi nguyên ý kiến; không gợi ý rằng vòng rẻ, bền hoặc đẹp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sau khi xem bộ thông tin</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Với mẫu, chất liệu/cỡ, giá và phí này, bạn chọn mẫu nào hoặc không chọn? Vì sao?</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Lưu đúng phiên bản đã xem; không loại phản hồi không muốn mua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Sau khi xem bộ thông tin</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Bạn sẽ chọn nhóm hay nơi khác? Điểm nào ảnh hưởng quyết định và điều gì cần thay đổi?</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Phân biệt giá trị khách cảm nhận với nhận xét nội bộ của nhóm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Khi nói về hành động</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Bạn có muốn đặt ở điều kiện đã thông báo không? Nếu có, thời điểm phù hợp là khi nào?</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Ý định, xác nhận đặt, tiền và giao nhận là các mức khác nhau; chỉ ghi trạng thái đã xảy ra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Có thể thử bán ở quy mô nhóm phê duyệt</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Mẫu/giá/điều kiện mua được xác nhận, phù hợp ngân sách; có cách cung ứng và khách được thông báo đúng điều kiện. Đây là điều kiện triển khai, chưa chứng minh sẽ có lãi.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Tiêu chí định tính đề xuất; chưa phải kết quả hoặc ngưỡng số đã được nhóm chốt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Giữ mẫu để kiểm tra tiếp</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Phản hồi chỉ ra mẫu/điều kiện phù hợp, có ý định cụ thể hoặc hành động mua được ghi nhận; đối chiếu cả lý do chọn và từ chối, chưa suy rộng thị trường.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu chí định tính đề xuất; chưa phải kết quả hoặc ngưỡng số đã được nhóm chốt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="85" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Điều chỉnh hoặc đổi phương án</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Khách không chọn vì mẫu, chất liệu/cỡ, giá/nhận hàng hoặc nguồn không đáp ứng điều kiện; ghi nguyên nhân và chỉ rõ thay đổi sẽ kiểm lại.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Tiêu chí định tính đề xuất; chưa phải kết quả hoặc ngưỡng số đã được nhóm chốt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="85" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đủ căn cứ kết luận</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Thiếu mẫu/giá xác nhận, chưa có phản hồi thực hoặc chỉ có tương tác mạng xã hội. Tiếp tục thu dữ liệu; không ghi đã thành công hoặc đã thất bại.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu chí định tính đề xuất; chưa phải kết quả hoặc ngưỡng số đã được nhóm chốt.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="70" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="65" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -1480,52 +1894,179 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Cách tuyển / kênh tiếp cận</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Lần đầu / khảo sát lại</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Mục đích mua</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Đã từng mua?</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Lần mua gần nhất</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Nơi mua thực tế tự khai</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Giá lịch sử tự khai</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Đơn vị chiếc / bộ / số lượng</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Ngân sách hỏi trước khi xem giá</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Mẫu đã xem / phiên bản</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Nguồn ảnh / mẫu thật</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Thông tin mẫu và giá đầy đủ đã xem</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Lựa chọn / không chọn</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Lý do chọn hoặc từ chối</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Ý định và thời điểm muốn mua</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Đồng ý ghi nhận / ghi chú</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="65" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mã đơn</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mã khách liên kết</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Thời điểm cập nhật</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mẫu / phiên bản đã xác nhận</t>
+        </is>
+      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Mẫu đã xem</t>
+          <t>Số chiếc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Nguồn ảnh / mẫu thật</t>
+          <t>Đơn giá / điều kiện combo</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Giá &amp; điều kiện đã thông báo</t>
+          <t>Tổng tiền hàng xác nhận</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Lựa chọn</t>
+          <t>Phí giao / người chịu</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Mức giá chấp nhận</t>
+          <t>Trạng thái hiện tại</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Lý do chọn / từ chối</t>
+          <t>Tiền đã nhận thực tế</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Hành động mua thực tế</t>
+          <t>Ngày giao thực tế</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Mã chứng từ nếu có</t>
+          <t>Lý do hủy / đổi nếu có</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Đồng ý ghi nhận / ghi chú</t>
+          <t>Link chứng từ / ghi chú</t>
         </is>
       </c>
     </row>
@@ -1533,4 +2074,157 @@
   <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="145" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mục</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nội dung cần làm rõ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Đầu mối đề xuất</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Tình trạng bằng chứng</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="85" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Khảo sát gốc</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Câu hỏi, phản hồi đã ẩn thông tin riêng, cách tuyển và địa bàn; làm rõ câu đơn/đa lựa chọn và phản hồi trùng.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Huy; Phong tổng hợp</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Chưa được cung cấp tệp gốc; có bản tổng hợp và link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="85" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tên Pinky / URL / giá</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Xác nhận 30.000đ/chiếc, 50.000đ/bộ 2 thuộc trang và cấu hình nào; lưu ảnh giá có ngày.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Huy/Danh</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Tài liệu dẫn hai tên miền; chưa được xác nhận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Giá Imoon và mức so sánh</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Link sản phẩm gốc, cấu hình/chất liệu, đơn vị giá, thời điểm và điều kiện bán nếu dùng làm đối chiếu.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Huy/Danh</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Nguồn hiện là trang shop trên ShopeeAnalytics; ba mẫu cùng một shop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Nguồn cung cho mẫu nhóm</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Báo giá ở lượng mua thực, vật liệu/cỡ, MOQ, phí và tồn; xác minh lại giới hạn nhập với đề/quyết định nhóm.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Bằng/Hưng; Nghĩa chốt</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Giá và điều kiện đơn nhỏ chưa được xác nhận trong đầu vào.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Triển khai tuần 2</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Xác nhận đầu mối, mẫu/giá dùng thử, tiêu chí và cách ghi dữ liệu; sau thực hiện lưu kết quả và quyết định.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Các Lead; Nghĩa chốt</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Mới có kế hoạch đề xuất; chưa có phản hồi/đơn tuần 2 được cung cấp.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>